<commit_message>
Atualização do codeVersion android para 30
</commit_message>
<xml_diff>
--- a/Documentação/promotion_codes.xlsx
+++ b/Documentação/promotion_codes.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Antonio\ArqReactNative\CalculadoraEletricaResidencial\documentacao\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Antonio\ArqReactNative\CalcEletrResidencial\Documentação\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="79">
   <si>
     <t>Promotion code</t>
   </si>
@@ -253,6 +253,9 @@
   </si>
   <si>
     <t>Ayrton (amigo do Vicente)</t>
+  </si>
+  <si>
+    <t>Zé Luiz Ópera</t>
   </si>
 </sst>
 </file>
@@ -1287,6 +1290,9 @@
       <c r="A29" t="s">
         <v>29</v>
       </c>
+      <c r="E29" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">

</xml_diff>